<commit_message>
Pertes bière : onglet XLSX « Sources & conventions » (pièce auto-justifiante)
Ajoute au RF-pertes-biere-mousse.xlsx un 3e onglet listant les conventions de
part bière (panaché/monaco 12,5 cl, Picon 23/46 cl), les taux de freinte
(7/8/5 % = 20 %), la fourchette documentée et les 5 sources avec leur URL.
La page conserve la pièce jointe + les liens sources cliquables.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/RF-pertes-biere-mousse.xlsx
+++ b/public/documents/pieces-defense/RF-pertes-biere-mousse.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Biere servie par article" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Freinte par exercice" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sources &amp; conventions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -986,4 +987,284 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Pertes de biere pression - freinte technique du fut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Biere pression servie par produit et par exercice, puis freinte technique (sur-versement/collerette, mousse &amp; tirage, nettoyage des lignes + purge + fond). Freinte retenue 20 % du fut (moyenne sectorielle, Modern Restaurant Management), au-dessus des 15 % du service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Detail / Source (lien)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>CONVENTIONS DE PART BIERE</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pression 25 cl / 50 cl</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Part biere = contenance (biere pure) : 25 cl / 50 cl</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Panache 25 cl</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Part biere 12,5 cl (moitie biere + limonade)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Monaco 25 cl</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Part biere 12,5 cl (biere + limonade + trait de grenadine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Picon biere 25 cl</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Part biere 23 cl (2 cl de Picon)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Picon biere 50 cl</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Part biere 46 cl (4 cl de Picon)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Distinction 25/50 cl</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Lue sur l'article de caisse (insensible au prix, qui varie par periode)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>TAUX DE FREINTE (% du fut tire)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Sur-versement / collerette</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>7 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mousse &amp; tirage (temperature, pression, debut/fond de fut)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>8 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Nettoyage des lignes + purge + fond de fut</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>5 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Total freinte retenue</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>20 % du fut = 305 L sur 3 ans</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Fourchette documentee</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>5 % a 25 %, moyenne ~20 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Retranche par le service (fisc)</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>15 % (Proposition p. 51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>SOURCES</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Modern Restaurant Management (moyenne 20 %/fut ; mousse = 25 % de biere)</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>https://modernrestaurantmanagement.com/seven-wasteful-sins-how-youre-losing-profits-on-draft-beer-sales/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Bar-i (fourchette 5-25 % ; moussage &gt; 10 %)</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>https://blog.bar-i.com/what-is-the-normal-waste-level-for-draft-beer</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Brewers Association - Draught Beer Quality Manual (nettoyage lignes / 14 jours)</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.brewersassociation.org/educational-publications/draught-beer-quality-manual/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Le Bihan Boissons - CHR France (~10 %/fut)</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>https://lebihanboissons.com/tirage-pression-comment-choisir-ses-futs-et-eviter-la-perte-mousse-stockage-service/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>JDC - CHR France (~15 %)</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jdc.fr/blog/reduire-gaspillage-de-biere-bar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>